<commit_message>
added ADOU basin, changed selector for advanced search button
</commit_message>
<xml_diff>
--- a/nexis_scraper/basins_searchterms_tracking.xlsx
+++ b/nexis_scraper/basins_searchterms_tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shared Waters Lab\geography\geography\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shared Waters Lab\nexis_scraper\nexis_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078C5ED3-2F15-4036-966B-51EF1414E398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A24DB1B-8DFE-4AEA-A498-246319550A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="754" yWindow="754" windowWidth="16457" windowHeight="8632" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="1112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="1115">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -3359,6 +3359,15 @@
   </si>
   <si>
     <t>Pakchan OR "Kra Buri" OR Kraburi OR "maenam kaburi" OR "Bamakgyi Chaung" OR kyaungwakyaung OR "K Hat khai tou"</t>
+  </si>
+  <si>
+    <t>ADOU</t>
+  </si>
+  <si>
+    <t>Adour</t>
+  </si>
+  <si>
+    <t>Adour OR "Gave de Pau" OR "La Nive" OR "La Bidouze" OR "La Douze" OR "La Midouze" OR "Le Luy" OR "Gave d'Oloron" OR Arros OR "Luy de Béarn" OR "Luy de France" OR Aran OR Estampon OR Gabas OR Ouzom OR Midour OR "Nive des Aldudes" OR Lihoury OR Louts OR Lées OR Midou OR "Gave d'Ossau" OR "Gaves Réunis" OR Lauribar OR "Luzaide ibaia" OR "Le Bès" OR "Adour de Gripp" OR Bastan OR "Gave de Cauterets" OR "Gave de Héas" OR "Gave du Marcadau" OR Ispatchoury OR "La Baïse" OR "Lakako erreka" OR "Le Bas" OR "Le Laâ" OR "Le Luz" OR Échez OR "Adour de Lesponne" OR Bouès OR Béez OR Estrigon OR "Gave d'Arrens" OR "Gave de Gavarnie" OR "La Joyeuse" OR "La Nive / Errobi" OR "La Nive d'Arnéguy" OR "Le Nés" OR Ardanabie OR Ardanavy OR Arriutort OR Bahus OR Bario OR "Bras du Gave d'Oloron" OR Estéous OR "Gave d'Aspe" OR "Gave d'Azun" OR "Gave d'Ossou" OR "Gave du Brousset" OR "Gave d’Ossau" OR Jarras OR Jouanin OR Lagoin OR "Las Hies" OR "Latsa ibaia" OR Neez OR "Ousse des Bois" OR Ousse OR Oussouet OR Pesqué OR d'Estiraux OR "Ühaïtxa erreka" OR Arcis OR Cabanes OR Geloux OR "La Gouaneyre" OR Luzou OR "Urritzateko erreka" OR "Anguéluko Erreka" OR "Aranteko erreka" OR Ayguette OR Batanès OR Bergons OR Cazeaux OR Esqueda OR Gioulé OR "Grand Arrigan" OR "Haltzabaltzako erreka" OR "Hosta Ur Handia" OR L'Uby OR "La Barthe Ouverte" OR "La Génie Longue" OR "Lakako Erreka" OR Lescle OR Lespontès OR "Lohitzeko erreka" OR Mardaing OR Moulin OR Mouréaou OR "Nive des Aldudes / Urepeleko Errobi" OR Ouzente OR Padescaux OR Retjons OR Saget OR Urhandia OR "la Gouaougue" OR "Adour d'Arizes" OR "Adour du Tourmalet" OR Alems OR Allier OR Anou OR "Arrec de Groute" OR Arribères OR Arrigan OR "Arriou Grand" OR Arrêt OR Arrêt-Darré OR Aube OR Aule OR Avezaguet OR Barats OR Barbe OR Baron OR Barran OR Barrancous OR Barry OR Barthes OR "Bastan de Sers" OR Batnère OR Bayet OR Bergon OR Bernazau OR Biarré OR Bidaudos OR "Biduze / La Bidouze" OR Bitet OR Brouilh OR Broussau OR Carbouère OR Cassagnet OR Castaings OR Caudia OR Cavaillon OR Christian OR Clamondé OR Corbleu OR Cosme OR Courrèges OR Cros OR "Eiheraxaharreko Erreka" OR Escou OR Estang OR Gabarret OR "Garraldako erreka" OR "Gave d'Aspé" OR "Gave de Cestrède" OR "Gaznategiko erreka" OR "Goua de Hourcq" OR Gouarde OR Graves OR Grècq OR Hontines OR Houndarré OR "Ihitiko erreka" OR Jeanchouaou OR Kehut OR "La Bardolle" OR "La Chella" OR "La Douloustre" OR "La Gespe" OR "La Geune" OR "La Géline" OR "La Juscle" OR "La Laque" OR "La Souye" OR Labésiau OR Laca OR Ladournan OR Laguibaou OR Laminosine OR Lanénos OR Larcis OR Larrazieu OR Larritou OR Lataillade OR Latsa OR Laudon OR Layet OR Laüs OR "Le Geü" OR Lenet OR Lesgouret OR Lies OR Louet OR Loumné OR Lourdén OR Lurus OR "Marmaroko erreka" OR Marrein OR Martinet OR Mauhé OR "Mendihaltzuko erreka" OR "Minhurièta erreka" OR Mollevielle OR "Moulin d'Esbouc" OR "Moulin de Bordes" OR "Moulin du Leuy" OR Moulins OR Noët OR "Orellako erreka / Gorritxuko erreka" OR "Otxinen erreka" OR "Petit Lées" OR "Pla de la Pène" OR "Pont du Sac" OR Portou OR Poustagnac OR Poustagnacq OR Pouy OR Saint-Pastous OR Serres OR Turré OR "Txorizako erreka" OR Vergoignan OR Vialote OR d'Arrimoula OR "d'Aygue Pich" OR d'Herrès OR d'Éstéré OR "de Tos" OR "du Mas" OR l'Artiguette OR l'Ousse OR l'Uzerte OR "la Grabe" OR "la Géline" OR "la Moulie" OR Marsan OR Cassagnac OR Uzerte OR l'Escourre OR Balaing OR "Péglé (Recouvert)" OR d'Alaric OR "la Traverse"</t>
   </si>
 </sst>
 </file>
@@ -3724,13 +3733,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G315"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G316"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="82.69140625" customWidth="1"/>
+    <col min="4" max="4" width="82.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3753,7 +3762,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3773,7 +3782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3793,7 +3802,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3813,7 +3822,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3833,7 +3842,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3853,7 +3862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3873,7 +3882,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3893,7 +3902,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3913,7 +3922,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3933,7 +3942,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3953,7 +3962,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3973,7 +3982,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="72.900000000000006" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3993,7 +4002,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
@@ -4013,7 +4022,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>13</v>
       </c>
@@ -4033,7 +4042,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
@@ -4053,7 +4062,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>15</v>
       </c>
@@ -4073,7 +4082,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>16</v>
       </c>
@@ -4093,7 +4102,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>17</v>
       </c>
@@ -4113,7 +4122,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>18</v>
       </c>
@@ -4133,7 +4142,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>19</v>
       </c>
@@ -4153,7 +4162,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>20</v>
       </c>
@@ -4173,7 +4182,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>21</v>
       </c>
@@ -4193,7 +4202,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>22</v>
       </c>
@@ -4213,7 +4222,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>23</v>
       </c>
@@ -4233,7 +4242,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>24</v>
       </c>
@@ -4253,7 +4262,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>25</v>
       </c>
@@ -4273,7 +4282,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>26</v>
       </c>
@@ -4293,7 +4302,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>27</v>
       </c>
@@ -4313,7 +4322,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>28</v>
       </c>
@@ -4333,7 +4342,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>29</v>
       </c>
@@ -4353,7 +4362,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>30</v>
       </c>
@@ -4373,7 +4382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>31</v>
       </c>
@@ -4393,7 +4402,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>32</v>
       </c>
@@ -4413,7 +4422,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>33</v>
       </c>
@@ -4433,7 +4442,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="72.900000000000006" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>34</v>
       </c>
@@ -4453,7 +4462,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>35</v>
       </c>
@@ -4473,7 +4482,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>36</v>
       </c>
@@ -4493,7 +4502,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>37</v>
       </c>
@@ -4513,7 +4522,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>38</v>
       </c>
@@ -4533,7 +4542,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>39</v>
       </c>
@@ -4553,7 +4562,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>40</v>
       </c>
@@ -4573,7 +4582,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>41</v>
       </c>
@@ -4593,7 +4602,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>42</v>
       </c>
@@ -4613,7 +4622,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>43</v>
       </c>
@@ -4633,7 +4642,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>44</v>
       </c>
@@ -4653,7 +4662,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>45</v>
       </c>
@@ -4673,7 +4682,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>46</v>
       </c>
@@ -4693,7 +4702,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>47</v>
       </c>
@@ -4713,7 +4722,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>48</v>
       </c>
@@ -4733,7 +4742,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>49</v>
       </c>
@@ -4753,7 +4762,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>50</v>
       </c>
@@ -4773,7 +4782,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>51</v>
       </c>
@@ -4793,7 +4802,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>52</v>
       </c>
@@ -4813,7 +4822,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="160.30000000000001" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>53</v>
       </c>
@@ -4833,7 +4842,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>54</v>
       </c>
@@ -4853,7 +4862,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>55</v>
       </c>
@@ -4873,7 +4882,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>56</v>
       </c>
@@ -4893,7 +4902,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>57</v>
       </c>
@@ -4913,7 +4922,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>58</v>
       </c>
@@ -4933,7 +4942,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>59</v>
       </c>
@@ -4953,7 +4962,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>60</v>
       </c>
@@ -4973,7 +4982,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="409.6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>61</v>
       </c>
@@ -4993,7 +5002,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>62</v>
       </c>
@@ -5013,7 +5022,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>63</v>
       </c>
@@ -5033,7 +5042,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="409.6" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>64</v>
       </c>
@@ -5053,7 +5062,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="409.6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A67">
         <v>65</v>
       </c>
@@ -5073,7 +5082,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="409.6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A68">
         <v>66</v>
       </c>
@@ -5093,7 +5102,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A69">
         <v>67</v>
       </c>
@@ -5113,7 +5122,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>68</v>
       </c>
@@ -5133,7 +5142,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="364.3" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:7" ht="342" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>69</v>
       </c>
@@ -5153,7 +5162,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>70</v>
       </c>
@@ -5173,7 +5182,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="409.6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A73">
         <v>71</v>
       </c>
@@ -5193,7 +5202,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>72</v>
       </c>
@@ -5213,7 +5222,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>73</v>
       </c>
@@ -5233,7 +5242,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>74</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>75</v>
       </c>
@@ -5273,7 +5282,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A78">
         <v>76</v>
       </c>
@@ -5293,7 +5302,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>77</v>
       </c>
@@ -5313,7 +5322,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>78</v>
       </c>
@@ -5333,7 +5342,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>79</v>
       </c>
@@ -5353,7 +5362,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>80</v>
       </c>
@@ -5373,7 +5382,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A83">
         <v>81</v>
       </c>
@@ -5393,7 +5402,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>82</v>
       </c>
@@ -5413,7 +5422,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A85">
         <v>83</v>
       </c>
@@ -5433,7 +5442,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A86">
         <v>84</v>
       </c>
@@ -5453,7 +5462,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A87">
         <v>85</v>
       </c>
@@ -5473,7 +5482,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A88">
         <v>86</v>
       </c>
@@ -5493,7 +5502,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A89">
         <v>87</v>
       </c>
@@ -5513,7 +5522,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A90">
         <v>88</v>
       </c>
@@ -5533,7 +5542,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A91">
         <v>89</v>
       </c>
@@ -5553,7 +5562,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A92">
         <v>90</v>
       </c>
@@ -5573,7 +5582,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A93">
         <v>91</v>
       </c>
@@ -5593,7 +5602,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A94">
         <v>92</v>
       </c>
@@ -5613,7 +5622,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A95">
         <v>93</v>
       </c>
@@ -5633,7 +5642,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A96">
         <v>94</v>
       </c>
@@ -5653,7 +5662,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A97">
         <v>95</v>
       </c>
@@ -5673,7 +5682,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A98">
         <v>96</v>
       </c>
@@ -5693,7 +5702,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A99">
         <v>97</v>
       </c>
@@ -5713,7 +5722,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A100">
         <v>98</v>
       </c>
@@ -5733,7 +5742,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A101">
         <v>99</v>
       </c>
@@ -5753,7 +5762,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A102">
         <v>100</v>
       </c>
@@ -5773,7 +5782,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A103">
         <v>101</v>
       </c>
@@ -5793,7 +5802,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A104">
         <v>102</v>
       </c>
@@ -5813,7 +5822,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A105">
         <v>103</v>
       </c>
@@ -5833,7 +5842,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A106">
         <v>104</v>
       </c>
@@ -5853,7 +5862,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A107">
         <v>105</v>
       </c>
@@ -5873,7 +5882,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A108">
         <v>106</v>
       </c>
@@ -5893,7 +5902,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A109">
         <v>107</v>
       </c>
@@ -5913,7 +5922,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A110">
         <v>108</v>
       </c>
@@ -5933,7 +5942,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A111">
         <v>109</v>
       </c>
@@ -5953,7 +5962,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A112">
         <v>110</v>
       </c>
@@ -5973,7 +5982,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A113">
         <v>111</v>
       </c>
@@ -5993,7 +6002,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A114">
         <v>112</v>
       </c>
@@ -6013,7 +6022,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A115">
         <v>113</v>
       </c>
@@ -6033,7 +6042,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A116">
         <v>114</v>
       </c>
@@ -6053,7 +6062,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A117">
         <v>115</v>
       </c>
@@ -6073,7 +6082,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A118">
         <v>116</v>
       </c>
@@ -6093,7 +6102,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A119">
         <v>117</v>
       </c>
@@ -6113,7 +6122,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A120">
         <v>118</v>
       </c>
@@ -6133,7 +6142,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A121">
         <v>119</v>
       </c>
@@ -6153,7 +6162,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A122">
         <v>120</v>
       </c>
@@ -6173,7 +6182,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A123">
         <v>121</v>
       </c>
@@ -6193,7 +6202,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A124">
         <v>122</v>
       </c>
@@ -6213,7 +6222,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A125">
         <v>123</v>
       </c>
@@ -6233,7 +6242,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A126">
         <v>124</v>
       </c>
@@ -6253,7 +6262,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A127">
         <v>125</v>
       </c>
@@ -6273,7 +6282,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A128">
         <v>126</v>
       </c>
@@ -6293,7 +6302,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A129">
         <v>127</v>
       </c>
@@ -6313,7 +6322,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A130">
         <v>128</v>
       </c>
@@ -6333,7 +6342,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A131">
         <v>129</v>
       </c>
@@ -6353,7 +6362,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A132">
         <v>130</v>
       </c>
@@ -6373,7 +6382,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A133">
         <v>131</v>
       </c>
@@ -6393,7 +6402,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A134">
         <v>132</v>
       </c>
@@ -6413,7 +6422,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A135">
         <v>133</v>
       </c>
@@ -6433,7 +6442,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A136">
         <v>134</v>
       </c>
@@ -6453,7 +6462,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A137">
         <v>135</v>
       </c>
@@ -6473,7 +6482,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A138">
         <v>136</v>
       </c>
@@ -6493,7 +6502,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A139">
         <v>137</v>
       </c>
@@ -6513,7 +6522,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A140">
         <v>138</v>
       </c>
@@ -6533,7 +6542,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A141">
         <v>139</v>
       </c>
@@ -6553,7 +6562,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A142">
         <v>140</v>
       </c>
@@ -6573,7 +6582,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A143">
         <v>141</v>
       </c>
@@ -6593,7 +6602,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A144">
         <v>142</v>
       </c>
@@ -6613,7 +6622,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A145">
         <v>143</v>
       </c>
@@ -6633,7 +6642,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A146">
         <v>144</v>
       </c>
@@ -6653,7 +6662,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A147">
         <v>145</v>
       </c>
@@ -6673,7 +6682,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A148">
         <v>146</v>
       </c>
@@ -6693,7 +6702,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A149">
         <v>147</v>
       </c>
@@ -6713,7 +6722,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A150">
         <v>148</v>
       </c>
@@ -6733,7 +6742,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A151">
         <v>149</v>
       </c>
@@ -6753,7 +6762,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A152">
         <v>150</v>
       </c>
@@ -6773,7 +6782,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A153">
         <v>151</v>
       </c>
@@ -6793,7 +6802,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A154">
         <v>152</v>
       </c>
@@ -6813,7 +6822,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A155">
         <v>153</v>
       </c>
@@ -6833,7 +6842,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A156">
         <v>154</v>
       </c>
@@ -6853,7 +6862,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A157">
         <v>155</v>
       </c>
@@ -6873,7 +6882,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A158">
         <v>156</v>
       </c>
@@ -6893,7 +6902,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A159">
         <v>157</v>
       </c>
@@ -6913,7 +6922,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A160">
         <v>158</v>
       </c>
@@ -6933,7 +6942,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A161">
         <v>159</v>
       </c>
@@ -6953,7 +6962,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A162">
         <v>160</v>
       </c>
@@ -6973,7 +6982,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A163">
         <v>161</v>
       </c>
@@ -6993,7 +7002,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A164">
         <v>162</v>
       </c>
@@ -7013,7 +7022,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A165">
         <v>163</v>
       </c>
@@ -7033,7 +7042,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A166">
         <v>164</v>
       </c>
@@ -7053,7 +7062,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A167">
         <v>165</v>
       </c>
@@ -7073,7 +7082,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A168">
         <v>166</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A169">
         <v>167</v>
       </c>
@@ -7113,7 +7122,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A170">
         <v>168</v>
       </c>
@@ -7133,7 +7142,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A171">
         <v>169</v>
       </c>
@@ -7153,7 +7162,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A172">
         <v>170</v>
       </c>
@@ -7173,7 +7182,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A173">
         <v>171</v>
       </c>
@@ -7193,7 +7202,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A174">
         <v>172</v>
       </c>
@@ -7213,7 +7222,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A175">
         <v>173</v>
       </c>
@@ -7233,7 +7242,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A176">
         <v>174</v>
       </c>
@@ -7253,7 +7262,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A177">
         <v>175</v>
       </c>
@@ -7273,7 +7282,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A178">
         <v>176</v>
       </c>
@@ -7293,7 +7302,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A179">
         <v>177</v>
       </c>
@@ -7313,7 +7322,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A180">
         <v>178</v>
       </c>
@@ -7333,7 +7342,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A181">
         <v>179</v>
       </c>
@@ -7353,7 +7362,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A182">
         <v>180</v>
       </c>
@@ -7373,7 +7382,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A183">
         <v>181</v>
       </c>
@@ -7393,7 +7402,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A184">
         <v>182</v>
       </c>
@@ -7413,7 +7422,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A185">
         <v>183</v>
       </c>
@@ -7433,7 +7442,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A186">
         <v>184</v>
       </c>
@@ -7453,7 +7462,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A187">
         <v>185</v>
       </c>
@@ -7473,7 +7482,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A188">
         <v>186</v>
       </c>
@@ -7493,7 +7502,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A189">
         <v>187</v>
       </c>
@@ -7513,7 +7522,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A190">
         <v>188</v>
       </c>
@@ -7533,7 +7542,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A191">
         <v>189</v>
       </c>
@@ -7553,7 +7562,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A192">
         <v>190</v>
       </c>
@@ -7573,7 +7582,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A193">
         <v>191</v>
       </c>
@@ -7593,7 +7602,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A194">
         <v>192</v>
       </c>
@@ -7613,7 +7622,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A195">
         <v>193</v>
       </c>
@@ -7633,7 +7642,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A196">
         <v>194</v>
       </c>
@@ -7653,7 +7662,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A197">
         <v>195</v>
       </c>
@@ -7673,7 +7682,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A198">
         <v>196</v>
       </c>
@@ -7693,7 +7702,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A199">
         <v>197</v>
       </c>
@@ -7713,7 +7722,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A200">
         <v>198</v>
       </c>
@@ -7733,7 +7742,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A201">
         <v>199</v>
       </c>
@@ -7753,7 +7762,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A202">
         <v>200</v>
       </c>
@@ -7773,7 +7782,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A203">
         <v>201</v>
       </c>
@@ -7793,7 +7802,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A204">
         <v>202</v>
       </c>
@@ -7813,7 +7822,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A205">
         <v>203</v>
       </c>
@@ -7833,7 +7842,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A206">
         <v>204</v>
       </c>
@@ -7853,7 +7862,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A207">
         <v>205</v>
       </c>
@@ -7873,7 +7882,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A208">
         <v>206</v>
       </c>
@@ -7893,7 +7902,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A209">
         <v>207</v>
       </c>
@@ -7913,7 +7922,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A210">
         <v>208</v>
       </c>
@@ -7933,7 +7942,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A211">
         <v>209</v>
       </c>
@@ -7953,7 +7962,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A212">
         <v>210</v>
       </c>
@@ -7973,7 +7982,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A213">
         <v>211</v>
       </c>
@@ -7993,7 +8002,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A214">
         <v>212</v>
       </c>
@@ -8013,7 +8022,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A215">
         <v>213</v>
       </c>
@@ -8033,7 +8042,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A216">
         <v>214</v>
       </c>
@@ -8053,7 +8062,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A217">
         <v>215</v>
       </c>
@@ -8073,7 +8082,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A218">
         <v>216</v>
       </c>
@@ -8093,7 +8102,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A219">
         <v>217</v>
       </c>
@@ -8113,7 +8122,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A220">
         <v>218</v>
       </c>
@@ -8133,7 +8142,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A221">
         <v>219</v>
       </c>
@@ -8153,7 +8162,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A222">
         <v>220</v>
       </c>
@@ -8173,7 +8182,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A223">
         <v>221</v>
       </c>
@@ -8193,7 +8202,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A224">
         <v>222</v>
       </c>
@@ -8213,7 +8222,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A225">
         <v>223</v>
       </c>
@@ -8233,7 +8242,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A226">
         <v>224</v>
       </c>
@@ -8253,7 +8262,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A227">
         <v>225</v>
       </c>
@@ -8273,7 +8282,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A228">
         <v>226</v>
       </c>
@@ -8293,7 +8302,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A229">
         <v>227</v>
       </c>
@@ -8313,7 +8322,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A230">
         <v>228</v>
       </c>
@@ -8333,7 +8342,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A231">
         <v>229</v>
       </c>
@@ -8353,7 +8362,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A232">
         <v>230</v>
       </c>
@@ -8373,7 +8382,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A233">
         <v>231</v>
       </c>
@@ -8393,7 +8402,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A234">
         <v>232</v>
       </c>
@@ -8413,7 +8422,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A235">
         <v>233</v>
       </c>
@@ -8433,7 +8442,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A236">
         <v>234</v>
       </c>
@@ -8453,7 +8462,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A237">
         <v>235</v>
       </c>
@@ -8473,7 +8482,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A238">
         <v>236</v>
       </c>
@@ -8493,7 +8502,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A239">
         <v>237</v>
       </c>
@@ -8513,7 +8522,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A240">
         <v>238</v>
       </c>
@@ -8533,7 +8542,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A241">
         <v>239</v>
       </c>
@@ -8553,7 +8562,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A242">
         <v>240</v>
       </c>
@@ -8573,7 +8582,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A243">
         <v>241</v>
       </c>
@@ -8593,7 +8602,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A244">
         <v>242</v>
       </c>
@@ -8613,7 +8622,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A245">
         <v>243</v>
       </c>
@@ -8633,7 +8642,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A246">
         <v>244</v>
       </c>
@@ -8653,7 +8662,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A247">
         <v>245</v>
       </c>
@@ -8673,7 +8682,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A248">
         <v>246</v>
       </c>
@@ -8693,7 +8702,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A249">
         <v>247</v>
       </c>
@@ -8713,7 +8722,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A250">
         <v>248</v>
       </c>
@@ -8733,7 +8742,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A251">
         <v>249</v>
       </c>
@@ -8753,7 +8762,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A252">
         <v>250</v>
       </c>
@@ -8773,7 +8782,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A253">
         <v>251</v>
       </c>
@@ -8793,7 +8802,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A254">
         <v>252</v>
       </c>
@@ -8813,7 +8822,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A255">
         <v>253</v>
       </c>
@@ -8833,7 +8842,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A256">
         <v>254</v>
       </c>
@@ -8853,7 +8862,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A257">
         <v>255</v>
       </c>
@@ -8873,7 +8882,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A258">
         <v>256</v>
       </c>
@@ -8893,7 +8902,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A259">
         <v>257</v>
       </c>
@@ -8913,7 +8922,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A260">
         <v>258</v>
       </c>
@@ -8933,7 +8942,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A261">
         <v>259</v>
       </c>
@@ -8953,7 +8962,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A262">
         <v>260</v>
       </c>
@@ -8973,7 +8982,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A263">
         <v>261</v>
       </c>
@@ -8993,7 +9002,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A264">
         <v>262</v>
       </c>
@@ -9013,7 +9022,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A265">
         <v>263</v>
       </c>
@@ -9033,7 +9042,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A266">
         <v>264</v>
       </c>
@@ -9053,7 +9062,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A267">
         <v>265</v>
       </c>
@@ -9073,7 +9082,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A268">
         <v>266</v>
       </c>
@@ -9093,7 +9102,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A269">
         <v>267</v>
       </c>
@@ -9113,7 +9122,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A270">
         <v>268</v>
       </c>
@@ -9133,7 +9142,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A271">
         <v>269</v>
       </c>
@@ -9153,7 +9162,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A272">
         <v>270</v>
       </c>
@@ -9173,7 +9182,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A273">
         <v>271</v>
       </c>
@@ -9193,7 +9202,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A274">
         <v>272</v>
       </c>
@@ -9213,7 +9222,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A275">
         <v>273</v>
       </c>
@@ -9233,7 +9242,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A276">
         <v>274</v>
       </c>
@@ -9253,7 +9262,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A277">
         <v>275</v>
       </c>
@@ -9273,7 +9282,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A278">
         <v>276</v>
       </c>
@@ -9293,7 +9302,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A279">
         <v>277</v>
       </c>
@@ -9313,7 +9322,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A280">
         <v>278</v>
       </c>
@@ -9333,7 +9342,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A281">
         <v>279</v>
       </c>
@@ -9353,7 +9362,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A282">
         <v>280</v>
       </c>
@@ -9373,7 +9382,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A283">
         <v>281</v>
       </c>
@@ -9393,7 +9402,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A284">
         <v>282</v>
       </c>
@@ -9413,7 +9422,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A285">
         <v>283</v>
       </c>
@@ -9433,7 +9442,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A286">
         <v>284</v>
       </c>
@@ -9453,7 +9462,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A287">
         <v>285</v>
       </c>
@@ -9473,7 +9482,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A288">
         <v>286</v>
       </c>
@@ -9493,7 +9502,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A289">
         <v>287</v>
       </c>
@@ -9513,7 +9522,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A290">
         <v>288</v>
       </c>
@@ -9533,7 +9542,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A291">
         <v>289</v>
       </c>
@@ -9553,7 +9562,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A292">
         <v>290</v>
       </c>
@@ -9573,7 +9582,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A293">
         <v>291</v>
       </c>
@@ -9593,7 +9602,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A294">
         <v>292</v>
       </c>
@@ -9613,7 +9622,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A295">
         <v>293</v>
       </c>
@@ -9633,7 +9642,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A296">
         <v>294</v>
       </c>
@@ -9653,7 +9662,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A297">
         <v>295</v>
       </c>
@@ -9673,7 +9682,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A298">
         <v>296</v>
       </c>
@@ -9693,7 +9702,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A299">
         <v>297</v>
       </c>
@@ -9713,7 +9722,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A300">
         <v>298</v>
       </c>
@@ -9733,7 +9742,7 @@
         <v>1038</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A301">
         <v>299</v>
       </c>
@@ -9753,7 +9762,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A302">
         <v>300</v>
       </c>
@@ -9773,7 +9782,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A303">
         <v>301</v>
       </c>
@@ -9793,7 +9802,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A304">
         <v>302</v>
       </c>
@@ -9813,7 +9822,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A305">
         <v>303</v>
       </c>
@@ -9833,7 +9842,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A306">
         <v>304</v>
       </c>
@@ -9853,7 +9862,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A307">
         <v>305</v>
       </c>
@@ -9873,7 +9882,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A308">
         <v>306</v>
       </c>
@@ -9893,7 +9902,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A309">
         <v>307</v>
       </c>
@@ -9913,7 +9922,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A310">
         <v>308</v>
       </c>
@@ -9933,7 +9942,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="311" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A311">
         <v>309</v>
       </c>
@@ -9953,7 +9962,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="312" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A312">
         <v>310</v>
       </c>
@@ -9973,7 +9982,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A313">
         <v>311</v>
       </c>
@@ -9993,7 +10002,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="314" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A314">
         <v>312</v>
       </c>
@@ -10013,7 +10022,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="315" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A315">
         <v>313</v>
       </c>
@@ -10028,6 +10037,26 @@
       </c>
       <c r="E315" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A316">
+        <v>314</v>
+      </c>
+      <c r="B316" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C316" t="s">
+        <v>1113</v>
+      </c>
+      <c r="D316" t="s">
+        <v>1114</v>
+      </c>
+      <c r="E316" t="s">
+        <v>10</v>
+      </c>
+      <c r="G316" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>